<commit_message>
production version of "harris-ahad"
</commit_message>
<xml_diff>
--- a/src/test/resources/bulk/image_manifest.xlsx
+++ b/src/test/resources/bulk/image_manifest.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="21075" windowHeight="10035"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="21930" windowHeight="6000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -21,9 +22,6 @@
     <t>5127663428_42ef7f4463_b.jpg</t>
   </si>
   <si>
-    <t>handbook_of_archaeology.jpg</t>
-  </si>
-  <si>
     <t>filename</t>
   </si>
   <si>
@@ -91,6 +89,9 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>HANDBOOK_of_archaeology.jpg</t>
   </si>
 </sst>
 </file>
@@ -108,17 +109,20 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -458,40 +462,43 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
       <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="G1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>15</v>
-      </c>
       <c r="K1" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -502,62 +509,62 @@
         <v>1234</v>
       </c>
       <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="K2" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B3">
         <v>2222</v>
       </c>
       <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
       <c r="E3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="K3" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>